<commit_message>
06g: a fixture a spreadsheet app opens, and the one-strike question at once
xlsxOf now writes the package's content types and a styles part with what
Excel expects, so hollis-mill.xlsx, regenerated, opens in a spreadsheet app;
a test checks every part has a content type. The one-strike stop shows as
soon as "No" is picked, warrant columns are asked too, and a made holder's
note questions put its name in quotes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dashboard/test/fixtures/hollis-mill.xlsx
+++ b/apps/dashboard/test/fixtures/hollis-mill.xlsx
@@ -422,10 +422,39 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0"/>
-    <xf numFmtId="14"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
 </styleSheet>
 </file>
 

</xml_diff>